<commit_message>
Changes to separate bid file upload process to include rebates and capacity
</commit_message>
<xml_diff>
--- a/tests/data/test_scenarios/test_1/separate/test_baseline.xlsx
+++ b/tests/data/test_scenarios/test_1/separate/test_baseline.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/peyton_wates_gapac_com/Documents/Documents/Ad hoc/RFP Analysis Automation Files/OneDrive_2024-09-16/RFP Submissions/RFP data test/Dummy data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chrisw78\RFP Automation REPO\RFP_Analysis_Automation2\tests\data\test_scenarios\test_1\separate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{B14F32EB-DBFB-4461-96D4-C65AD6D5B2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EA1058B-ACA1-4D8E-A8C5-1241EAD8E525}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2B09322-7D75-443D-95CD-1AEC312C3AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{968BBE7F-5A2B-4921-8F1D-9AB52A9A3C3A}"/>
+    <workbookView xWindow="9060" yWindow="7080" windowWidth="28665" windowHeight="12360" activeTab="2" xr2:uid="{968BBE7F-5A2B-4921-8F1D-9AB52A9A3C3A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="rebates" sheetId="2" r:id="rId2"/>
+    <sheet name="capacity" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t>Bid ID</t>
   </si>
@@ -89,22 +91,49 @@
     <t>B</t>
   </si>
   <si>
-    <t>Supplier 1</t>
-  </si>
-  <si>
-    <t>Supplier 6</t>
-  </si>
-  <si>
-    <t>Supplier 7</t>
-  </si>
-  <si>
-    <t>Supplier 4</t>
-  </si>
-  <si>
-    <t>Supplier 2</t>
-  </si>
-  <si>
     <t>Current Price</t>
+  </si>
+  <si>
+    <t>Chris</t>
+  </si>
+  <si>
+    <t>Minia</t>
+  </si>
+  <si>
+    <t>Amber</t>
+  </si>
+  <si>
+    <t>Jared</t>
+  </si>
+  <si>
+    <t>Peyton</t>
+  </si>
+  <si>
+    <t>Supplier Name</t>
+  </si>
+  <si>
+    <t>Min Volume</t>
+  </si>
+  <si>
+    <t>Max Volume</t>
+  </si>
+  <si>
+    <t>Min Spend</t>
+  </si>
+  <si>
+    <t>Max Spend</t>
+  </si>
+  <si>
+    <t>% Rebate</t>
+  </si>
+  <si>
+    <t>$ Rebate</t>
+  </si>
+  <si>
+    <t>Grouping</t>
+  </si>
+  <si>
+    <t>Capacity</t>
   </si>
 </sst>
 </file>
@@ -114,10 +143,25 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -143,9 +187,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,7 +564,7 @@
         <v>3</v>
       </c>
       <c r="H1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -533,7 +581,7 @@
         <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2">
         <v>3437457</v>
@@ -637,7 +685,7 @@
         <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F6">
         <v>45000</v>
@@ -647,6 +695,66 @@
       </c>
       <c r="H6" s="1">
         <v>0.35700000000000004</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="GUID" r:id="rId1"/>
+  </customProperties>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54B9E7A3-9D21-48C3-BAA5-FFC427E65DF5}">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <customProperties>
+    <customPr name="GUID" r:id="rId1"/>
+  </customProperties>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03FABEA2-70A3-429A-9407-97BB02387BE9}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>